<commit_message>
Update kaspa_buys.xlsx after running on 2026-09-18
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D57"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1346,6 +1346,22 @@
         <v>25</v>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>09/18/2026</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>729.6749999999956</v>
+      </c>
+      <c r="C58" t="n">
+        <v>0.03391921060746243</v>
+      </c>
+      <c r="D58" t="n">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-09-25
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:D59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1362,6 +1362,22 @@
         <v>25</v>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>09/25/2026</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>614.7419999999984</v>
+      </c>
+      <c r="C59" t="n">
+        <v>0.04026079233239321</v>
+      </c>
+      <c r="D59" t="n">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-10-02
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:D60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1378,6 +1378,22 @@
         <v>25</v>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>10/02/2026</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>1185.824999999997</v>
+      </c>
+      <c r="C60" t="n">
+        <v>0.041743090253621</v>
+      </c>
+      <c r="D60" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-10-09
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D60"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1394,6 +1394,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>1246.307000000001</v>
+      </c>
+      <c r="C61" t="n">
+        <v>0.03971734091199036</v>
+      </c>
+      <c r="D61" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-10-16
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1410,6 +1410,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>10/16/2026</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>1362.03300000001</v>
+      </c>
+      <c r="C62" t="n">
+        <v>0.03634273178403138</v>
+      </c>
+      <c r="D62" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-10-23
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1426,6 +1426,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>10/23/2026</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>1328.803999999989</v>
+      </c>
+      <c r="C63" t="n">
+        <v>0.03725154349324687</v>
+      </c>
+      <c r="D63" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-10-30
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1442,6 +1442,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>10/30/2026</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>1412.667999999998</v>
+      </c>
+      <c r="C64" t="n">
+        <v>0.03504008018869265</v>
+      </c>
+      <c r="D64" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>